<commit_message>
chore(sync): E8 local xlsx re-save (openpyxl byte-sync, 0 content changes)
All 9 E8 corrected cells verified identical on remote (cleancheck snapshot).
Byte diff is openpyxl internal metadata only.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excels/8_asses.masses_E8Proxy.xlsx
+++ b/excels/8_asses.masses_E8Proxy.xlsx
@@ -226,13 +226,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="0000B050"/>
+      </left>
+      <right style="thin">
+        <color rgb="0000B050"/>
+      </right>
+      <top style="thin">
+        <color rgb="0000B050"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0000B050"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -423,6 +437,12 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -29165,7 +29185,7 @@
           <t>Yazık. Çiftlik'teki günlerden sonra çok hızlı bir değişimdi!</t>
         </is>
       </c>
-      <c r="J17" s="36" t="inlineStr">
+      <c r="J17" s="66" t="inlineStr">
         <is>
           <t>Oh, jammer. Het was een leuke afwisseling van de dagen op de Hoeve!</t>
         </is>
@@ -43058,7 +43078,7 @@
           <t>Kullar, buraya gelmekte oldukça geciktiniz.</t>
         </is>
       </c>
-      <c r="J6" s="53" t="inlineStr">
+      <c r="J6" s="67" t="inlineStr">
         <is>
           <t>Vazallen, Uw aanwezigheid is bijzonder achterstallig.</t>
         </is>
@@ -43522,7 +43542,7 @@
           <t>Hafızanızı sileceğiz ki Ruh'unuz sorunsuzca yeni bir Eşek'e can verebilsin.</t>
         </is>
       </c>
-      <c r="J14" s="53" t="inlineStr">
+      <c r="J14" s="67" t="inlineStr">
         <is>
           <t>Wij zullen Uw herinneringen wissen, opdat Uw Ziel ongehinderd een nieuw Ezellichaam kan binnentreden.</t>
         </is>
@@ -43580,7 +43600,7 @@
           <t>Reeşekkarnasyon için hazırlanın.</t>
         </is>
       </c>
-      <c r="J15" s="53" t="inlineStr">
+      <c r="J15" s="67" t="inlineStr">
         <is>
           <t>Bereid U voor op Heraanstelling.</t>
         </is>
@@ -43990,7 +44010,7 @@
           <t xml:space="preserve">Ruh'unun Reeşekkarnasyon'a girmemesine karar verdik. </t>
         </is>
       </c>
-      <c r="J22" s="53" t="inlineStr">
+      <c r="J22" s="67" t="inlineStr">
         <is>
           <t>Wij hebben besloten dat Uw Ziel geen Heraanstelling zal ondergaan.</t>
         </is>
@@ -44628,7 +44648,7 @@
           <t>Seninle birlikte çalışmayı ve bu üzücü durumu düzeltmeyi sabırsızlıkla bekliyoruz.</t>
         </is>
       </c>
-      <c r="J33" s="53" t="inlineStr">
+      <c r="J33" s="67" t="inlineStr">
         <is>
           <t>Wij zien ernaar uit met U samen te werken en deze droevige toestand te herstellen.</t>
         </is>
@@ -45042,7 +45062,7 @@
           <t>Hayır, Ruh'un bir daha asla Reeşekkarnasyon'a girmeyecek.</t>
         </is>
       </c>
-      <c r="J40" s="53" t="inlineStr">
+      <c r="J40" s="67" t="inlineStr">
         <is>
           <t>Neen, Uw Ziel zal nooit meer Heraanstelling ondergaan.</t>
         </is>
@@ -45162,7 +45182,7 @@
           <t>Hizmetlerin için teşekkür ederiz.</t>
         </is>
       </c>
-      <c r="J42" s="53" t="inlineStr">
+      <c r="J42" s="67" t="inlineStr">
         <is>
           <t>Wij danken U voor Uw dienst.</t>
         </is>
@@ -45224,7 +45244,7 @@
           <t>Tarılar'la bir olmak için hazırlan.</t>
         </is>
       </c>
-      <c r="J43" s="53" t="inlineStr">
+      <c r="J43" s="67" t="inlineStr">
         <is>
           <t>Bereid U voor om één te worden met Uw Goden.</t>
         </is>

</xml_diff>